<commit_message>
give F1 room to breathe and the PCA some ellipses
</commit_message>
<xml_diff>
--- a/04_Figures/F1/c_data/F1.xlsx
+++ b/04_Figures/F1/c_data/F1.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="902" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="363">
   <si>
     <t>sheet</t>
   </si>
@@ -878,6 +878,12 @@
   </si>
   <si>
     <t>4.0.3</t>
+  </si>
+  <si>
+    <t>ggrepel</t>
+  </si>
+  <si>
+    <t>0.9.8</t>
   </si>
   <si>
     <t>ggtext</t>
@@ -6403,7 +6409,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -6557,18 +6563,18 @@
         <v>285</v>
       </c>
       <c r="C14" t="s">
-        <v>286</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
+        <v>286</v>
+      </c>
+      <c r="B15" t="s">
         <v>287</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>288</v>
-      </c>
-      <c r="C15" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -6645,7 +6651,7 @@
         <v>302</v>
       </c>
       <c r="C22" t="s">
-        <v>286</v>
+        <v>261</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -6656,7 +6662,7 @@
         <v>304</v>
       </c>
       <c r="C23" t="s">
-        <v>261</v>
+        <v>288</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -6799,7 +6805,7 @@
         <v>330</v>
       </c>
       <c r="C36" t="s">
-        <v>286</v>
+        <v>261</v>
       </c>
     </row>
     <row r="37" spans="1:3">
@@ -6810,7 +6816,7 @@
         <v>332</v>
       </c>
       <c r="C37" t="s">
-        <v>261</v>
+        <v>288</v>
       </c>
     </row>
     <row r="38" spans="1:3">
@@ -6884,7 +6890,7 @@
         <v>345</v>
       </c>
       <c r="B44" t="s">
-        <v>308</v>
+        <v>346</v>
       </c>
       <c r="C44" t="s">
         <v>261</v>
@@ -6892,10 +6898,10 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B45" t="s">
-        <v>275</v>
+        <v>310</v>
       </c>
       <c r="C45" t="s">
         <v>261</v>
@@ -6903,10 +6909,10 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B46" t="s">
-        <v>348</v>
+        <v>275</v>
       </c>
       <c r="C46" t="s">
         <v>261</v>
@@ -6975,6 +6981,17 @@
         <v>360</v>
       </c>
       <c r="C52" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
+        <v>361</v>
+      </c>
+      <c r="B53" t="s">
+        <v>362</v>
+      </c>
+      <c r="C53" t="s">
         <v>261</v>
       </c>
     </row>

</xml_diff>

<commit_message>
teach every figure to save itself the same way
</commit_message>
<xml_diff>
--- a/04_Figures/F1/c_data/F1.xlsx
+++ b/04_Figures/F1/c_data/F1.xlsx
@@ -631,7 +631,7 @@
     <t>02_HRvLR/01_Protein_Contrasts/c_data/protein_contrasts.xlsx</t>
   </si>
   <si>
-    <t>e706deccf806204996a968b97f852521</t>
+    <t>eb23e8a1866fdf41427417935863def8</t>
   </si>
   <si>
     <t>variance</t>
@@ -649,7 +649,7 @@
     <t>02_HRvLR/07_Group_Trait_Slopes/c_data/group_trait_slopes.xlsx</t>
   </si>
   <si>
-    <t>f24590e2277ed08b7470c1cb8b4f4eee</t>
+    <t>6dd01c4da2455f99b603e6b8b9827643</t>
   </si>
   <si>
     <t>BiocManager</t>

</xml_diff>

<commit_message>
widen S1 and give its colour key a proper legend instead of hand-placed tiles
</commit_message>
<xml_diff>
--- a/04_Figures/F1/c_data/F1.xlsx
+++ b/04_Figures/F1/c_data/F1.xlsx
@@ -640,7 +640,7 @@
     <t>02_HRvLR/04_Variance/c_data/variance.xlsx</t>
   </si>
   <si>
-    <t>21f4207236305a5ac8a5be8a5cbaf4be</t>
+    <t>844320d78318f2e845c02f6db890b83d</t>
   </si>
   <si>
     <t>slopes</t>
@@ -649,7 +649,7 @@
     <t>02_HRvLR/07_Group_Trait_Slopes/c_data/group_trait_slopes.xlsx</t>
   </si>
   <si>
-    <t>6dd01c4da2455f99b603e6b8b9827643</t>
+    <t>f24590e2277ed08b7470c1cb8b4f4eee</t>
   </si>
   <si>
     <t>BiocManager</t>

</xml_diff>

<commit_message>
rebuild the modules coarser so most of them survive losing any one person
</commit_message>
<xml_diff>
--- a/04_Figures/F1/c_data/F1.xlsx
+++ b/04_Figures/F1/c_data/F1.xlsx
@@ -668,7 +668,7 @@
     <t>02_HRvLR/07_Group_Trait_Slopes/c_data/group_trait_slopes.xlsx</t>
   </si>
   <si>
-    <t>f24590e2277ed08b7470c1cb8b4f4eee</t>
+    <t>cd5d6ebfaf5bb2df64f241c5bc674e40</t>
   </si>
   <si>
     <t>set_tests</t>
@@ -677,7 +677,7 @@
     <t>02_HRvLR/02_Set_Contrasts/c_data/set_tests.rds</t>
   </si>
   <si>
-    <t>30db8bea525624e038076e732efccd5f</t>
+    <t>913e33734a82439181cc7dfdb9ea1917</t>
   </si>
   <si>
     <t>BiocManager</t>

</xml_diff>

<commit_message>
sweep out what nobody reads and correct the READMEs that miscounted
</commit_message>
<xml_diff>
--- a/04_Figures/F1/c_data/F1.xlsx
+++ b/04_Figures/F1/c_data/F1.xlsx
@@ -650,7 +650,7 @@
     <t>02_HRvLR/01_Protein_Contrasts/c_data/protein_contrasts.xlsx</t>
   </si>
   <si>
-    <t>eb23e8a1866fdf41427417935863def8</t>
+    <t>f1b9b3d5ee159b256de22fc2b72e89ce</t>
   </si>
   <si>
     <t>variance</t>
@@ -659,7 +659,7 @@
     <t>02_HRvLR/04_Variance/c_data/variance.xlsx</t>
   </si>
   <si>
-    <t>844320d78318f2e845c02f6db890b83d</t>
+    <t>f1ad3960759c75b00d78e1297f45e7ad</t>
   </si>
   <si>
     <t>slopes</t>
@@ -668,7 +668,7 @@
     <t>02_HRvLR/07_Group_Trait_Slopes/c_data/group_trait_slopes.xlsx</t>
   </si>
   <si>
-    <t>cd5d6ebfaf5bb2df64f241c5bc674e40</t>
+    <t>b2284ace62d57e411d12c11b4087bb9c</t>
   </si>
   <si>
     <t>set_tests</t>

</xml_diff>